<commit_message>
Đồng bộ hai website theo app bản 172: cột 7 sinh lại cả 51 cặp khối × môn (Tiếng Anh 4, Tiếng Việt 2, GDTC 4-5 hết lệch tên bài)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/docs/lop1/KHDH ca khoi - Lop 1.xlsx
+++ b/assets/docs/lop1/KHDH ca khoi - Lop 1.xlsx
@@ -16099,7 +16099,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -16168,7 +16168,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -16202,7 +16202,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -16237,7 +16237,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -16271,7 +16271,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -16306,7 +16306,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -16340,7 +16340,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -16375,7 +16375,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -16409,7 +16409,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -16444,7 +16444,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -16478,7 +16478,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -16513,7 +16513,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -16547,7 +16547,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -16581,7 +16581,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -16615,7 +16615,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -16645,7 +16645,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -16679,7 +16679,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -16709,7 +16709,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -16743,7 +16743,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -16777,7 +16777,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -16841,7 +16841,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -16876,7 +16876,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -16910,7 +16910,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -16944,7 +16944,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -16979,7 +16979,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -17013,7 +17013,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -17048,7 +17048,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -17082,7 +17082,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -17117,7 +17117,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -17151,7 +17151,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -17186,7 +17186,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -17220,7 +17220,7 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -17318,7 +17318,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -17353,7 +17353,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -17387,7 +17387,7 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -17422,7 +17422,7 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -17456,7 +17456,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -17491,7 +17491,7 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -17525,7 +17525,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -17560,7 +17560,7 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -17594,7 +17594,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -17629,7 +17629,7 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -17663,7 +17663,7 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -17698,7 +17698,7 @@
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -17732,7 +17732,7 @@
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -17766,7 +17766,7 @@
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -17796,7 +17796,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -17826,7 +17826,7 @@
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -17860,7 +17860,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -17894,7 +17894,7 @@
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -17924,7 +17924,7 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -17954,7 +17954,7 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -18022,7 +18022,7 @@
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -18056,7 +18056,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -18086,7 +18086,7 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -18116,7 +18116,7 @@
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -18150,7 +18150,7 @@
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -18214,7 +18214,7 @@
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -18244,7 +18244,7 @@
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -18274,7 +18274,7 @@
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -18308,7 +18308,7 @@
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">

</xml_diff>